<commit_message>
feat: synchronize visualizer DOM IDs, fix selftest diacritics & layout, generate Session 05 resources
</commit_message>
<xml_diff>
--- a/pms/PM_Python.xlsx
+++ b/pms/PM_Python.xlsx
@@ -426,7 +426,7 @@
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
@@ -516,27 +516,27 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Tổng quan về Python, lịch sử và ứng dụng thực tế</t>
+          <t>Tổng quan về Python, lịch sử và ứng dụng thực tế trong các lĩnh vực (Web, Data, Automation)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Hiểu rõ khái niệm và cấu trúc 01: Giới thiệu ngôn ngữ Python (Tổng quan về Python, lịch sử và ứng dụng thực tế); vận dụng tự viết và thực thi thành công mã nguồn/sản phẩm thực hành chuẩn kỹ thuật.</t>
+          <t>Giải thích được cơ chế hoạt động dạng thông dịch của Python, trình bày được lịch sử phát triển và liệt kê được ít nhất 3 lĩnh vực ứng dụng thực tế phổ biến của ngôn ngữ này.</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CẤM: Code phức tạp, Algorithm, Loop, Function, Class, Module, NumPy, Pandas.</t>
+          <t>CẤM: Khai báo biến, toán tử, vòng lặp, cấu trúc điều kiện, hàm, class và các thư viện NumPy/Pandas.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: Chưa có (Buổi mở đầu).</t>
+          <t>Chưa có (Buổi mở đầu).</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Python 3.12, VS Code, Virtual Env</t>
+          <t>python/core</t>
         </is>
       </c>
     </row>
@@ -568,27 +568,27 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Cài đặt Python, VS Code, Anaconda/Virtual Environment</t>
+          <t>Cài đặt Python, cấu hình biến môi trường toàn cục và thiết lập trình soạn thảo VS Code cùng môi trường ảo Virtual Environment</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Hiểu rõ khái niệm và cấu trúc 02: Cài đặt môi trường (Cài đặt Python, VS Code, Anaconda/Virtual Environment); vận dụng tự viết và thực thi thành công mã nguồn/sản phẩm thực hành chuẩn kỹ thuật.</t>
+          <t>Thiết lập thành công môi trường lập trình Python 3.12 trên máy tính cá nhân, cài đặt thành thạo IDE VS Code và kích hoạt được Virtual Environment qua Terminal.</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>CẤM: Code phức tạp, Algorithm, Loop, Function, Class, Module, NumPy, Pandas.</t>
+          <t>CẤM: Thực hiện lập trình logic phức tạp, vòng lặp, cấu trúc dữ liệu List/Dict, Class.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: Chưa có (Buổi mở đầu).</t>
+          <t>ĐÃ HỌC: Tổng quan về vị trí và ứng dụng của Python.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Python 3.12, VS Code, Virtual Env</t>
+          <t>python/core</t>
         </is>
       </c>
     </row>
@@ -620,27 +620,27 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Khái niệm biến, quy tắc đặt tên, gán giá trị</t>
+          <t>Khái niệm biến, quy tắc đặt tên chuẩn PEP 8 và phép gán giá trị</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Hiểu rõ khái niệm và cấu trúc 03: Khai báo Biến (Khái niệm biến, quy tắc đặt tên, gán giá trị); vận dụng tự viết và thực thi thành công mã nguồn/sản phẩm thực hành chuẩn kỹ thuật.</t>
+          <t>Khai báo và gán giá trị thành công cho các biến; viết chương trình gán thông tin cá nhân cơ bản và tuân thủ tuyệt đối quy tắc đặt tên Snake_case của PEP 8.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CẤM: Code phức tạp, Algorithm, Loop, Function, Class, Module, NumPy, Pandas.</t>
+          <t>CẤM: Kiểu dữ liệu phức tạp (List, Dict), cấu trúc điều kiện (if-else), vòng lặp, hàm.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: Chưa có (Buổi mở đầu).</t>
+          <t>ĐÃ HỌC: Môi trường lập trình Python, cách chạy file script qua terminal.</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Python 3.12, VS Code, Virtual Env</t>
+          <t>python/core</t>
         </is>
       </c>
     </row>

</xml_diff>